<commit_message>
feat: Adjust gap analysis threshold to include scores up to 2 and add a new skills resource file.
</commit_message>
<xml_diff>
--- a/resources/skills.xlsx
+++ b/resources/skills.xlsx
@@ -1,20 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lohan.silva\Documents\projetos\skillmap\skillmap\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18200" windowHeight="8510"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
   <si>
     <t>Colaborador</t>
   </si>
@@ -34,35 +39,70 @@
     <t>RPA</t>
   </si>
   <si>
-    <t xml:space="preserve">BotCity / Selenium </t>
-  </si>
-  <si>
     <t>Backend</t>
   </si>
   <si>
-    <t xml:space="preserve">Python / FastAPI </t>
-  </si>
-  <si>
     <t>Web</t>
   </si>
   <si>
     <t>TypeScript</t>
   </si>
   <si>
-    <t>Membro 2</t>
-  </si>
-  <si>
     <t>Cloud</t>
   </si>
   <si>
     <t>AWS (Deploy)</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>BotCity / Selenium</t>
+  </si>
+  <si>
+    <t>Processos</t>
+  </si>
+  <si>
+    <t>Mapeamento de Processos</t>
+  </si>
+  <si>
+    <t>Agile / Scrum</t>
+  </si>
+  <si>
+    <t>Hyperautomation</t>
+  </si>
+  <si>
+    <t>IA</t>
+  </si>
+  <si>
+    <t>IA / Agentes</t>
+  </si>
+  <si>
+    <t>FastAPI / Flask</t>
+  </si>
+  <si>
+    <t>Dados</t>
+  </si>
+  <si>
+    <t>SQL / DB</t>
+  </si>
+  <si>
+    <t>DevOps</t>
+  </si>
+  <si>
+    <t>Git / DevOps</t>
+  </si>
+  <si>
+    <t>NestJS</t>
+  </si>
+  <si>
+    <t>Angular</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -74,13 +114,13 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF1f1f1f"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF1f1f1f"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -118,59 +158,58 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FF000000"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="medium">
-        <color rgb="FF000000"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="medium">
-        <color rgb="FF000000"/>
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -181,10 +220,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -222,71 +261,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -314,7 +353,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -337,11 +376,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -350,13 +389,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -366,7 +405,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -375,7 +414,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -384,7 +423,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -392,10 +431,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -464,16 +503,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="3" width="13.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -487,63 +524,190 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="32.25" customFormat="1" s="1">
-      <c r="A2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="1" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="32.25" customFormat="1" s="1">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="1">
-      <c r="A4" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="D11" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D14" s="7">
         <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="32.25" customFormat="1" s="1">
-      <c r="A5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="7">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Feat: Add dockerfile and docker-compose
</commit_message>
<xml_diff>
--- a/resources/skills.xlsx
+++ b/resources/skills.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lohan.silva\Documents\projetos\skillmap\skillmap\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ausier.neto\Documents\Automation\skillmap\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="43">
   <si>
     <t>Colaborador</t>
   </si>
@@ -97,13 +97,64 @@
   </si>
   <si>
     <t>Angular</t>
+  </si>
+  <si>
+    <t>Ausier</t>
+  </si>
+  <si>
+    <t>FastAPI / Django</t>
+  </si>
+  <si>
+    <t>Agile / ScrumBan</t>
+  </si>
+  <si>
+    <t>SQL / PostgreSQL</t>
+  </si>
+  <si>
+    <t>Desktop</t>
+  </si>
+  <si>
+    <t>C# / WPF</t>
+  </si>
+  <si>
+    <t>Docker / CI/CD (GitLab)</t>
+  </si>
+  <si>
+    <t>TensorFlow / Keras</t>
+  </si>
+  <si>
+    <t>Data Science (Pandas/Numpy)</t>
+  </si>
+  <si>
+    <t>HTML / CSS</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>José Jorge Rodrigues Abrahim</t>
+  </si>
+  <si>
+    <t>HTML</t>
+  </si>
+  <si>
+    <t>CSS</t>
+  </si>
+  <si>
+    <t>JavaScript</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,10 +170,22 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -175,15 +238,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -192,12 +252,16 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -503,11 +567,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="13.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -520,7 +584,7 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -703,6 +767,426 @@
         <v>10</v>
       </c>
       <c r="D14" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D36" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D37" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D38" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D39" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D42" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D43" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="8">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Modify skill sheet to match the team stats
</commit_message>
<xml_diff>
--- a/resources/skills.xlsx
+++ b/resources/skills.xlsx
@@ -9,17 +9,18 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18200" windowHeight="8510"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18200" windowHeight="8510" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="80">
   <si>
     <t>Colaborador</t>
   </si>
@@ -141,20 +142,131 @@
     <t>José Jorge Rodrigues Abrahim</t>
   </si>
   <si>
-    <t>HTML</t>
-  </si>
-  <si>
-    <t>CSS</t>
-  </si>
-  <si>
     <t>JavaScript</t>
+  </si>
+  <si>
+    <t>HTML/CSS</t>
+  </si>
+  <si>
+    <t>Victor Brito</t>
+  </si>
+  <si>
+    <t>FastAPI</t>
+  </si>
+  <si>
+    <t>Banco de Dados</t>
+  </si>
+  <si>
+    <t>RestAPIs</t>
+  </si>
+  <si>
+    <t>NodeJs</t>
+  </si>
+  <si>
+    <t>Selenium</t>
+  </si>
+  <si>
+    <t>BotCity</t>
+  </si>
+  <si>
+    <t>Playwright</t>
+  </si>
+  <si>
+    <t>ETL</t>
+  </si>
+  <si>
+    <t>Dashboards</t>
+  </si>
+  <si>
+    <t>ML</t>
+  </si>
+  <si>
+    <t>Agentes</t>
+  </si>
+  <si>
+    <t>OCR (Optical Character Recognition)</t>
+  </si>
+  <si>
+    <t>IA Generativa</t>
+  </si>
+  <si>
+    <t>Bancos Vetoriais</t>
+  </si>
+  <si>
+    <t>Agile / Kanban</t>
+  </si>
+  <si>
+    <t>Git / Versionamento</t>
+  </si>
+  <si>
+    <t>Docker</t>
+  </si>
+  <si>
+    <t>Java (Android)</t>
+  </si>
+  <si>
+    <t>Kotlin</t>
+  </si>
+  <si>
+    <t>José Jorge</t>
+  </si>
+  <si>
+    <t>Victor</t>
+  </si>
+  <si>
+    <t>RPA Core</t>
+  </si>
+  <si>
+    <t>RPA / Hyperautomation</t>
+  </si>
+  <si>
+    <t>Frameworks Python (FastAPI/Django/Flask)</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Node.js / NestJS (Target Project)</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>TypeScript / JavaScript</t>
+  </si>
+  <si>
+    <t>SQL / Banco de Dados</t>
+  </si>
+  <si>
+    <t>Data Science / ETL / Pandas</t>
+  </si>
+  <si>
+    <t>Inteligência Artificial / ML / Agentes</t>
+  </si>
+  <si>
+    <t>CI/CD / Docker / Git</t>
+  </si>
+  <si>
+    <t>Gestão</t>
+  </si>
+  <si>
+    <t>Processos Ágeis (ScrumBan / Mapeamento)</t>
+  </si>
+  <si>
+    <t>AWS (Deploy/Infra)</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Skill</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,15 +297,43 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Google Sans Text"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Google Sans Text"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA6A6A6"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -205,32 +345,32 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
+      <left style="thin">
+        <color rgb="FF1F1F1F"/>
       </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
+      <right style="thin">
+        <color rgb="FF1F1F1F"/>
       </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
+      <top style="thin">
+        <color rgb="FF1F1F1F"/>
       </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
+      <bottom style="thin">
+        <color rgb="FF1F1F1F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -238,13 +378,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -252,16 +389,32 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,29 +720,29 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D74"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="3" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="13.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="6" t="s">
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1">
+      <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -602,8 +755,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1">
+      <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -616,8 +769,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="6" t="s">
@@ -630,8 +783,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="1" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:4" s="1" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -644,8 +797,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:4" s="1" customFormat="1" ht="32.25" customHeight="1">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -658,8 +811,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -672,8 +825,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -686,8 +839,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:4">
+      <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -700,8 +853,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:4">
+      <c r="A10" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -714,8 +867,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:4">
+      <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -728,8 +881,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:4">
+      <c r="A12" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -742,8 +895,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="6" t="s">
+    <row r="13" spans="1:4">
+      <c r="A13" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -756,8 +909,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:4">
+      <c r="A14" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -770,423 +923,843 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:4">
+      <c r="A15" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="B15" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="5" t="s">
+      <c r="D15" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28">
+      <c r="A16" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="B16" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="5" t="s">
+      <c r="D16" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28">
+      <c r="A17" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="5" t="s">
+      <c r="D17" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="28">
+      <c r="A18" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="5" t="s">
+      <c r="D18" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28">
+      <c r="A19" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="5" t="s">
+      <c r="D19" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="5" t="s">
+      <c r="D20" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="5" t="s">
+      <c r="D21" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="5" t="s">
+      <c r="D22" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="42">
+      <c r="A23" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="5" t="s">
+      <c r="D23" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="28">
+      <c r="A24" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D24" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="5" t="s">
+      <c r="D24" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="42">
+      <c r="A25" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D25" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="5" t="s">
+      <c r="D25" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D26" s="5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="5" t="s">
+      <c r="D26" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="5" t="s">
+      <c r="D27" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="1:4">
+      <c r="A29" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="8" t="s">
+    <row r="30" spans="1:4">
+      <c r="A30" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C30" s="8" t="s">
+      <c r="B30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="8" t="s">
+      <c r="D30" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C31" s="8" t="s">
+      <c r="B31" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D31" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="8" t="s">
+      <c r="D31" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D32" s="8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
+      <c r="D32" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D33" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="8" t="s">
+      <c r="D33" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C34" s="8" t="s">
+      <c r="B34" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="8" t="s">
+      <c r="D34" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="8">
+      <c r="D35" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="8" t="s">
+    <row r="36" spans="1:4">
+      <c r="A36" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D36" s="8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" s="8" t="s">
+      <c r="D36" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D37" s="8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" s="8" t="s">
+      <c r="D37" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D38" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D38" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" s="8" t="s">
+      <c r="D39" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B40" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C39" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D39" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" s="8" t="s">
+      <c r="C40" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B41" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C40" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D40" s="8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" s="8" t="s">
+      <c r="C41" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B42" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C42" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D42" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D44" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D46" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D47" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D49" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D50" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D41" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B42" s="8" t="s">
+      <c r="D51" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B52" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C52" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D52" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D53" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D42" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D43" s="8">
+      <c r="D54" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B44" s="8" t="s">
+    <row r="55" spans="1:4">
+      <c r="A55" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C55" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D55" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D57" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D58" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C59" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D59" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C60" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D60" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C61" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D61" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C62" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D62" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D63" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D64" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C65" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D65" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D66" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C67" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C68" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C69" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D69" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C70" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D70" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C71" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D71" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C72" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D72" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C73" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D73" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B74" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" s="8">
+      <c r="C74" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D74" s="11">
         <v>0</v>
       </c>
     </row>
@@ -1194,4 +1767,298 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="17.26953125" customWidth="1"/>
+    <col min="2" max="2" width="26.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="12">
+        <v>5</v>
+      </c>
+      <c r="D2" s="12">
+        <v>5</v>
+      </c>
+      <c r="E2" s="13">
+        <v>4</v>
+      </c>
+      <c r="F2" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="12">
+        <v>5</v>
+      </c>
+      <c r="D3" s="12">
+        <v>5</v>
+      </c>
+      <c r="E3" s="13">
+        <v>4</v>
+      </c>
+      <c r="F3" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="12">
+        <v>4</v>
+      </c>
+      <c r="D4" s="13">
+        <v>4</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="13">
+        <v>2</v>
+      </c>
+      <c r="D5" s="13">
+        <v>2</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="12">
+        <v>3</v>
+      </c>
+      <c r="D6" s="13">
+        <v>2</v>
+      </c>
+      <c r="E6" s="13">
+        <v>1</v>
+      </c>
+      <c r="F6" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="12">
+        <v>4</v>
+      </c>
+      <c r="D7" s="13">
+        <v>2</v>
+      </c>
+      <c r="E7" s="13">
+        <v>3</v>
+      </c>
+      <c r="F7" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="12">
+        <v>3</v>
+      </c>
+      <c r="D8" s="13">
+        <v>4</v>
+      </c>
+      <c r="E8" s="13">
+        <v>4</v>
+      </c>
+      <c r="F8" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="12">
+        <v>4</v>
+      </c>
+      <c r="D9" s="13">
+        <v>3</v>
+      </c>
+      <c r="E9" s="13">
+        <v>4</v>
+      </c>
+      <c r="F9" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="12">
+        <v>4</v>
+      </c>
+      <c r="D10" s="13">
+        <v>4</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="12">
+        <v>4</v>
+      </c>
+      <c r="D11" s="12">
+        <v>4</v>
+      </c>
+      <c r="E11" s="13">
+        <v>1</v>
+      </c>
+      <c r="F11" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="12">
+        <v>4</v>
+      </c>
+      <c r="D12" s="13">
+        <v>3</v>
+      </c>
+      <c r="E12" s="13">
+        <v>3</v>
+      </c>
+      <c r="F12" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="12">
+        <v>3</v>
+      </c>
+      <c r="D13" s="12">
+        <v>4</v>
+      </c>
+      <c r="E13" s="13">
+        <v>4</v>
+      </c>
+      <c r="F13" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="13">
+        <v>1</v>
+      </c>
+      <c r="D14" s="13">
+        <v>0</v>
+      </c>
+      <c r="E14" s="13">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>